<commit_message>
added exp 6 & 7
</commit_message>
<xml_diff>
--- a/EXP_6/READINGS/CLOSED_LOOP.xlsx
+++ b/EXP_6/READINGS/CLOSED_LOOP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EDC_LAB\EXP_6\READINGS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F05A7119-10C5-4395-8ED9-976778FF1452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CE091A3-70A3-4EB0-8999-4412A6F3AC7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0E27E477-AB99-47CD-9512-0BB61835DBD3}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
   <si>
     <t>UNITY GAIN</t>
   </si>
@@ -85,6 +85,12 @@
   </si>
   <si>
     <t xml:space="preserve">NO AC INPUT </t>
+  </si>
+  <si>
+    <t>VOUT1(mV</t>
+  </si>
+  <si>
+    <t>VIN(mV)</t>
   </si>
 </sst>
 </file>
@@ -2641,37 +2647,93 @@
   <dimension ref="A1:E36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C2">
+        <v>50</v>
+      </c>
+      <c r="D2">
+        <v>64</v>
+      </c>
+      <c r="E2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C3">
+        <v>150</v>
+      </c>
+      <c r="D3">
+        <v>168</v>
+      </c>
+      <c r="E3">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <v>300</v>
+      </c>
+      <c r="D4">
+        <v>304</v>
+      </c>
+      <c r="E4">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <v>400</v>
+      </c>
+      <c r="D5">
+        <v>400</v>
+      </c>
+      <c r="E5">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <v>500</v>
+      </c>
+      <c r="D6">
+        <v>512</v>
+      </c>
+      <c r="E6">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -2685,7 +2747,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>5</v>
       </c>
@@ -2699,7 +2761,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2713,7 +2775,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>50</v>
       </c>
@@ -2727,7 +2789,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>100</v>
       </c>
@@ -2741,7 +2803,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>200</v>
       </c>
@@ -2755,7 +2817,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>500</v>
       </c>
@@ -2769,7 +2831,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>700</v>
       </c>
@@ -2822,25 +2884,70 @@
       <c r="A21" t="s">
         <v>9</v>
       </c>
+      <c r="C21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>15</v>
       </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22">
+        <v>51.2</v>
+      </c>
+      <c r="E22">
+        <v>44</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>10</v>
       </c>
+      <c r="C23">
+        <v>20</v>
+      </c>
+      <c r="D23">
+        <v>164</v>
+      </c>
+      <c r="E23">
+        <v>160</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>11</v>
       </c>
+      <c r="C24">
+        <v>50</v>
+      </c>
+      <c r="D24">
+        <v>392</v>
+      </c>
+      <c r="E24">
+        <v>360</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>12</v>
+      </c>
+      <c r="C25">
+        <v>100</v>
+      </c>
+      <c r="D25">
+        <v>780</v>
+      </c>
+      <c r="E25">
+        <v>700</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>